<commit_message>
Anpassungen an den Selektoren vorgenommen, BeurteilungsIds im Flowchart an produktiv umgestellt
</commit_message>
<xml_diff>
--- a/dispatcher/Data/Config.xlsx
+++ b/dispatcher/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KM\KM6\KM61_neu\15_RPA\02 Beurteilungsdaten übertragen\rpa005_TBÜ_Dispatcher_v1\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KM\KM6\KM61_neu\15_RPA\02_Beurteilungsdaten_übertragen\repo\dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBAB3DD9-1229-4652-B553-86DAFDA0B677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE99C3D-0B73-405D-8504-C600CA867C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-53325" yWindow="2295" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="56">
   <si>
     <t>Name</t>
   </si>
@@ -159,55 +159,40 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
+    <t>rpa005_EmailSmtpPort</t>
+  </si>
+  <si>
+    <t>rpa005_EmailSmtpServer</t>
+  </si>
+  <si>
+    <t>rpa005_FTP_Client_Url</t>
+  </si>
+  <si>
+    <t>rpa005_JsonNewFolderPath</t>
+  </si>
+  <si>
+    <t>rpa005_JsonProcessedFolderPath</t>
+  </si>
+  <si>
+    <t>rpa005_JsonErrorFolderPath</t>
+  </si>
+  <si>
+    <t>rpa005_JsonDispatcherFolderPath</t>
+  </si>
+  <si>
+    <t>rpa005_ZipFile</t>
+  </si>
+  <si>
+    <t>rpa005_LogFileFolderPath</t>
+  </si>
+  <si>
+    <t>rpa005_Email_Exception_Mailbox</t>
+  </si>
+  <si>
+    <t>rpa005_Bot_Email_Address</t>
+  </si>
+  <si>
     <t>rpa005_Beurteilungsdaten_übertragen</t>
-  </si>
-  <si>
-    <t>TMS_FTP_CredentialAssetName</t>
-  </si>
-  <si>
-    <t>rpa005_TMS_FTP_Account</t>
-  </si>
-  <si>
-    <t>rpa005_EmailSmtpPort</t>
-  </si>
-  <si>
-    <t>rpa005_EmailSmtpServer</t>
-  </si>
-  <si>
-    <t>rpa005_FTP_Client_Url</t>
-  </si>
-  <si>
-    <t>Test/POR/rpa005_TBÜ</t>
-  </si>
-  <si>
-    <t>rpa005_JsonNewFolderPath</t>
-  </si>
-  <si>
-    <t>rpa005_JsonProcessedFolderPath</t>
-  </si>
-  <si>
-    <t>rpa005_JsonErrorFolderPath</t>
-  </si>
-  <si>
-    <t>rpa005_JsonDispatcherFolderPath</t>
-  </si>
-  <si>
-    <t>rpa005_ZipFile</t>
-  </si>
-  <si>
-    <t>rpa005_LogFileFolderPath</t>
-  </si>
-  <si>
-    <t>rpa005_TestGroup_Mailbox</t>
-  </si>
-  <si>
-    <t>rpa005_Test_VersandMail</t>
-  </si>
-  <si>
-    <t>POR_Robot_Account</t>
-  </si>
-  <si>
-    <t>RPA_Bot_CredentialAssetName</t>
   </si>
 </sst>
 </file>
@@ -660,7 +645,7 @@
         <v>24</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>22</v>
@@ -669,9 +654,6 @@
     <row r="3" spans="1:26" ht="45">
       <c r="A3" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>50</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>32</v>
@@ -690,20 +672,10 @@
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>46</v>
-      </c>
+      <c r="B6" s="3"/>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="B7" t="s">
-        <v>59</v>
-      </c>
+      <c r="B7"/>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
@@ -2862,7 +2834,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z995"/>
+  <dimension ref="A1:Z993"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="5" customWidth="1"/>
@@ -2910,106 +2882,106 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>51</v>
+      <c r="A6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>53</v>
+      <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" t="s">
-        <v>54</v>
+      <c r="A9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>56</v>
+      <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>58</v>
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A13" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" t="s">
-        <v>48</v>
+      <c r="A13" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" t="s">
-        <v>47</v>
-      </c>
-      <c r="B14" t="s">
-        <v>47</v>
+      <c r="A14" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
@@ -3991,10 +3963,9 @@
     <row r="991" ht="14.25" customHeight="1"/>
     <row r="992" ht="14.25" customHeight="1"/>
     <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
FTP Client Ordner leeren aktiviert, Asset korrigiert
</commit_message>
<xml_diff>
--- a/dispatcher/Data/Config.xlsx
+++ b/dispatcher/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KM\KM6\KM61_neu\15_RPA\02_Beurteilungsdaten_übertragen\repo\dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE99C3D-0B73-405D-8504-C600CA867C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7E4740-39D4-4C06-9B51-90E9C05F72D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-33450" yWindow="7200" windowWidth="25845" windowHeight="17025" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="57">
   <si>
     <t>Name</t>
   </si>
@@ -193,6 +193,9 @@
   </si>
   <si>
     <t>rpa005_Beurteilungsdaten_übertragen</t>
+  </si>
+  <si>
+    <t>rpa005_Email_Group_Mailbox</t>
   </si>
 </sst>
 </file>
@@ -1671,6 +1674,9 @@
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <customProperties>
+    <customPr name="_pios_id" r:id="rId2"/>
+  </customProperties>
 </worksheet>
 </file>
 
@@ -2829,6 +2835,9 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <customProperties>
+    <customPr name="_pios_id" r:id="rId1"/>
+  </customProperties>
 </worksheet>
 </file>
 
@@ -2984,7 +2993,14 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A15" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1"/>
     <row r="18" ht="14.25" customHeight="1"/>
@@ -3967,5 +3983,8 @@
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <customProperties>
+    <customPr name="_pios_id" r:id="rId2"/>
+  </customProperties>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added wait for Download in Download Folder
</commit_message>
<xml_diff>
--- a/dispatcher/Data/Config.xlsx
+++ b/dispatcher/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KM\KM6\KM61_neu\15_RPA\02_Beurteilungsdaten_übertragen\repo\dispatcher\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arthur.folz\Documents\GitHub_Repos\RPA_005_TBÜ\uipath-rpa_tbu\dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7E4740-39D4-4C06-9B51-90E9C05F72D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B53B362-77A6-48FC-AFA0-1B33A6E5305E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-33450" yWindow="7200" windowWidth="25845" windowHeight="17025" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Assestts in Config angepasst
</commit_message>
<xml_diff>
--- a/dispatcher/Data/Config.xlsx
+++ b/dispatcher/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arthur.folz\Documents\GitHub_Repos\RPA_005_TBÜ\uipath-rpa_tbu\dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B53B362-77A6-48FC-AFA0-1B33A6E5305E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3576579-A30C-4BC8-933D-8250934903A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-47775" yWindow="6705" windowWidth="23085" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="56">
   <si>
     <t>Name</t>
   </si>
@@ -184,9 +184,6 @@
   </si>
   <si>
     <t>rpa005_LogFileFolderPath</t>
-  </si>
-  <si>
-    <t>rpa005_Email_Exception_Mailbox</t>
   </si>
   <si>
     <t>rpa005_Bot_Email_Address</t>
@@ -648,7 +645,7 @@
         <v>24</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>22</v>
@@ -1855,7 +1852,7 @@
         <v>40</v>
       </c>
       <c r="B17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>42</v>
@@ -2843,7 +2840,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z993"/>
+  <dimension ref="A1:Z992"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="5" customWidth="1"/>
@@ -2987,20 +2984,13 @@
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A15" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1"/>
     <row r="18" ht="14.25" customHeight="1"/>
@@ -3978,7 +3968,6 @@
     <row r="990" ht="14.25" customHeight="1"/>
     <row r="991" ht="14.25" customHeight="1"/>
     <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>